<commit_message>
In user API agent parameter added
</commit_message>
<xml_diff>
--- a/API URLs.xlsx
+++ b/API URLs.xlsx
@@ -153,6 +153,69 @@
   </si>
   <si>
     <t>{
+  "email": "vinod21@spidergang.com",
+  "password": "123456"
+}</t>
+  </si>
+  <si>
+    <t>{
+  "amount": "10000",
+  "type": "Home Loan",
+  "agent_name": "Vinod Nardiya",
+  "rate_of_interest": "14.99",
+  "duration": "1 Year"
+}</t>
+  </si>
+  <si>
+    <t>{
+  "amount": "20000",
+  "type": "Home Loan",
+  "agent_name": "Vinod Nardiya",
+  "rate_of_interest": "14.99",
+  "duration": "2 Year"
+}</t>
+  </si>
+  <si>
+    <t>{
+  "amount": "20000",
+  "type": "Car Insurance",
+  "agent_name": "Vinod Nardiya 2",
+  "duration": "2 Year"
+}</t>
+  </si>
+  <si>
+    <t>{
+  "amount": "10000",
+  "time": "17:54:23",
+  "from_account": "Vinod Nardiya",
+  "to_account": "AB Nardiya"
+}</t>
+  </si>
+  <si>
+    <t>{
+  "amount": "10000",
+  "time": "17:54:26",
+  "from_account": "Vinod Nardiya 12",
+  "to_account": "AAB Nardiya"
+}</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>insurance autoincrement id at end of url</t>
+  </si>
+  <si>
+    <t>loan auto increment id at end of URL</t>
+  </si>
+  <si>
+    <t>transaction auto increment id at end of url</t>
+  </si>
+  <si>
+    <t>{
   "name": "Vinod Nardiya",
   "email": "vinod21@spidergang.com",
   "phone": "9650236245",
@@ -161,71 +224,8 @@
   "password": "123456",
   "confirm_password": "123456",
   "dob": "2019-04-21",
-  "address": "this is valid address"
+  "address": "this is valid address","agent":"No"
 }</t>
-  </si>
-  <si>
-    <t>{
-  "email": "vinod21@spidergang.com",
-  "password": "123456"
-}</t>
-  </si>
-  <si>
-    <t>{
-  "amount": "10000",
-  "type": "Home Loan",
-  "agent_name": "Vinod Nardiya",
-  "rate_of_interest": "14.99",
-  "duration": "1 Year"
-}</t>
-  </si>
-  <si>
-    <t>{
-  "amount": "20000",
-  "type": "Home Loan",
-  "agent_name": "Vinod Nardiya",
-  "rate_of_interest": "14.99",
-  "duration": "2 Year"
-}</t>
-  </si>
-  <si>
-    <t>{
-  "amount": "20000",
-  "type": "Car Insurance",
-  "agent_name": "Vinod Nardiya 2",
-  "duration": "2 Year"
-}</t>
-  </si>
-  <si>
-    <t>{
-  "amount": "10000",
-  "time": "17:54:23",
-  "from_account": "Vinod Nardiya",
-  "to_account": "AB Nardiya"
-}</t>
-  </si>
-  <si>
-    <t>{
-  "amount": "10000",
-  "time": "17:54:26",
-  "from_account": "Vinod Nardiya 12",
-  "to_account": "AAB Nardiya"
-}</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>Comments</t>
-  </si>
-  <si>
-    <t>insurance autoincrement id at end of url</t>
-  </si>
-  <si>
-    <t>loan auto increment id at end of URL</t>
-  </si>
-  <si>
-    <t>transaction auto increment id at end of url</t>
   </si>
 </sst>
 </file>
@@ -589,7 +589,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="165" x14ac:dyDescent="0.25">
@@ -606,7 +606,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -621,7 +621,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -653,7 +653,7 @@
         <v>9</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="105" x14ac:dyDescent="0.25">
@@ -668,10 +668,10 @@
         <v>26</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -685,7 +685,7 @@
         <v>27</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -699,7 +699,7 @@
         <v>10</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -719,7 +719,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="90" x14ac:dyDescent="0.25">
@@ -734,10 +734,10 @@
         <v>26</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -752,7 +752,7 @@
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -784,7 +784,7 @@
         <v>9</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="90" x14ac:dyDescent="0.25">
@@ -799,10 +799,10 @@
         <v>26</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -817,7 +817,7 @@
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>